<commit_message>
Add PWA support and local reminders; fix day tabs and login UX
PWA: manifest.json, service worker (network-first with offline cache
fallback), and generated app icons (scripts/generate-icons.js, fixing
a sharp bug where .flatten() after an SVG-sourced resize wiped the
whole canvas to a solid color).

Notifications: local reminders 15 minutes before each of a
participant's events, capped at a 20-day scheduling window (setTimeout
overflows past ~24.8 days) and re-armed on visibility change. Includes
a permission banner and a temporary manual test button on the
Informacje page (marked for removal in stage 6).

Fixes: day-tab pills in Agenda/Moje aktywności now update their active
state on click instead of only scrolling. Login now requires an
explicit "Jazda" button after picking a name instead of logging in
immediately on selection, and the name filter matches by prefix
instead of substring.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Event_Data.xlsx
+++ b/data/Event_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fortedigital-my.sharepoint.com/personal/patrycja_galczynska_fortedigital_com/Documents/company-event-app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="612" documentId="8_{A2B12678-4492-5343-A762-7DCAF82DF857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E948FA2-4886-4942-B858-FA4931206BA6}"/>
+  <xr:revisionPtr revIDLastSave="617" documentId="8_{A2B12678-4492-5343-A762-7DCAF82DF857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA8DD305-2A68-BC4A-B5EB-907160ADB4D5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{8B06E614-3048-1B47-8A2C-EDAF591299DD}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" xr2:uid="{8B06E614-3048-1B47-8A2C-EDAF591299DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Agenda" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="267">
   <si>
     <t>ID</t>
   </si>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>Lunch przed wyjazdem, we własnym zakresie</t>
-  </si>
-  <si>
-    <t>Przejazd do hotelu i check-in. Prosimy o punktualność na miejscu zbiórki (ul. Krupnicza 3)</t>
   </si>
   <si>
     <t>Czas wolny w hotelu</t>
@@ -843,6 +840,12 @@
   </si>
   <si>
     <t>Marcin Ko</t>
+  </si>
+  <si>
+    <t>Przejazd do hotelu i check-in</t>
+  </si>
+  <si>
+    <t>Prosimy o punktualność na miejscu zbiórki (ul. Krupnicza 3)</t>
   </si>
 </sst>
 </file>
@@ -1304,7 +1307,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
@@ -1336,7 +1339,7 @@
         <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G2" t="s">
         <v>18</v>
@@ -1345,10 +1348,10 @@
         <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -1365,19 +1368,22 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>265</v>
       </c>
       <c r="F3" t="s">
-        <v>79</v>
+        <v>78</v>
+      </c>
+      <c r="G3" t="s">
+        <v>266</v>
       </c>
       <c r="H3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -1394,22 +1400,22 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>22</v>
       </c>
       <c r="I4" t="s">
         <v>17</v>
       </c>
       <c r="J4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -1426,22 +1432,22 @@
         <v>0.875</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I5" t="s">
         <v>17</v>
       </c>
       <c r="J5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -1458,22 +1464,22 @@
         <v>0.875</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I6" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="J6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -1490,22 +1496,22 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I7" t="s">
         <v>17</v>
       </c>
       <c r="J7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1522,22 +1528,22 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I8" t="s">
         <v>17</v>
       </c>
       <c r="J8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -1554,22 +1560,22 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I9" t="s">
         <v>17</v>
       </c>
       <c r="J9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -1586,22 +1592,22 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I10" t="s">
         <v>17</v>
       </c>
       <c r="J10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -1618,22 +1624,22 @@
         <v>0.9375</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I11" t="s">
         <v>17</v>
       </c>
       <c r="J11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -1641,7 +1647,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C12" s="1">
         <v>0.3125</v>
@@ -1650,22 +1656,22 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="E12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I12" t="s">
         <v>17</v>
       </c>
       <c r="J12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -1673,7 +1679,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C13" s="1">
         <v>0.33333333333333331</v>
@@ -1682,22 +1688,22 @@
         <v>0.875</v>
       </c>
       <c r="E13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I13" t="s">
         <v>17</v>
       </c>
       <c r="J13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1705,7 +1711,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C14" s="1">
         <v>0.375</v>
@@ -1714,22 +1720,22 @@
         <v>0.875</v>
       </c>
       <c r="E14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I14" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="J14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -1737,7 +1743,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C15" s="1">
         <v>0.39583333333333331</v>
@@ -1746,22 +1752,22 @@
         <v>0.5625</v>
       </c>
       <c r="E15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G15" t="s">
         <v>5</v>
       </c>
       <c r="H15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -1769,7 +1775,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C16" s="1">
         <v>0.5625</v>
@@ -1778,22 +1784,22 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="E16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
         <v>5</v>
       </c>
       <c r="H16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -1801,7 +1807,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C17" s="1">
         <v>0.58333333333333337</v>
@@ -1813,19 +1819,19 @@
         <v>15</v>
       </c>
       <c r="F17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G17" t="s">
         <v>5</v>
       </c>
       <c r="H17" t="s">
+        <v>50</v>
+      </c>
+      <c r="I17" t="s">
+        <v>41</v>
+      </c>
+      <c r="J17" t="s">
         <v>51</v>
-      </c>
-      <c r="I17" t="s">
-        <v>42</v>
-      </c>
-      <c r="J17" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -1833,7 +1839,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C18" s="1">
         <v>0.625</v>
@@ -1842,22 +1848,22 @@
         <v>0.65625</v>
       </c>
       <c r="E18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G18" t="s">
         <v>5</v>
       </c>
       <c r="H18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -1865,7 +1871,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C19" s="1">
         <v>0.6875</v>
@@ -1874,22 +1880,22 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="E19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G19" t="s">
         <v>5</v>
       </c>
       <c r="H19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
@@ -1897,7 +1903,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C20" s="1">
         <v>0.77083333333333337</v>
@@ -1906,22 +1912,22 @@
         <v>0.77430555555555558</v>
       </c>
       <c r="E20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G20" t="s">
         <v>5</v>
       </c>
       <c r="H20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I20" t="s">
         <v>17</v>
       </c>
       <c r="J20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -1929,7 +1935,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C21" s="1">
         <v>0.77083333333333337</v>
@@ -1938,22 +1944,22 @@
         <v>0.125</v>
       </c>
       <c r="E21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G21" t="s">
         <v>5</v>
       </c>
       <c r="H21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I21" t="s">
         <v>17</v>
       </c>
       <c r="J21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
@@ -1961,7 +1967,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C22" s="1">
         <v>0.3125</v>
@@ -1970,22 +1976,22 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="E22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I22" t="s">
         <v>17</v>
       </c>
       <c r="J22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -1993,7 +1999,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C23" s="1">
         <v>0.33333333333333331</v>
@@ -2002,22 +2008,22 @@
         <v>0.875</v>
       </c>
       <c r="E23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I23" t="s">
         <v>17</v>
       </c>
       <c r="J23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -2025,7 +2031,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C24" s="1">
         <v>0.375</v>
@@ -2034,22 +2040,22 @@
         <v>0.875</v>
       </c>
       <c r="E24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I24" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="J24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -2057,7 +2063,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C25" s="1">
         <v>0.39583333333333331</v>
@@ -2066,22 +2072,22 @@
         <v>0.5</v>
       </c>
       <c r="E25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I25" t="s">
         <v>17</v>
       </c>
       <c r="J25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -2089,7 +2095,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C26" s="1">
         <v>0.4375</v>
@@ -2098,22 +2104,22 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="E26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I26" t="s">
         <v>17</v>
       </c>
       <c r="J26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2132,13 +2138,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
         <v>5</v>
@@ -2146,122 +2152,122 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>17</v>
@@ -2272,10 +2278,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>17</v>
@@ -2286,10 +2292,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>17</v>
@@ -2300,10 +2306,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>17</v>
@@ -2314,13 +2320,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -2328,13 +2334,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -2342,13 +2348,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -2356,13 +2362,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -2370,10 +2376,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>17</v>
@@ -2384,10 +2390,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>17</v>
@@ -2398,13 +2404,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
         <v>5</v>
@@ -2412,13 +2418,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
@@ -2426,12 +2432,12 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2459,749 +2465,749 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" t="s">
         <v>85</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>86</v>
-      </c>
-      <c r="E1" t="s">
-        <v>87</v>
       </c>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C29" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C31" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C32" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C35" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C38" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C42" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C43" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C44" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C45" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C48" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C49" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C50" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C51" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C52" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C53" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C55" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C56" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C57" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C58" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C59" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C60" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C61" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C62" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C63" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C64" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C65" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -3235,7 +3241,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>9</v>
@@ -3250,18 +3256,18 @@
         <v>3</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
         <v>14</v>
@@ -3273,21 +3279,21 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="G2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" s="1">
         <v>0.5</v>
@@ -3296,21 +3302,21 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="G3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E4" s="1">
         <v>0.5</v>
@@ -3319,143 +3325,143 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="G4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3492,15 +3498,15 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
@@ -3508,23 +3514,23 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B8" s="10">
         <v>48579642504</v>
@@ -3532,15 +3538,15 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B10" s="11">
         <v>48737308331</v>
@@ -3548,15 +3554,15 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B13" s="1">
         <v>0.45833333333333331</v>
@@ -3564,34 +3570,34 @@
     </row>
     <row r="16" spans="1:2" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>184</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>185</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>186</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>187</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>